<commit_message>
Complete Wise valuation analysis
</commit_message>
<xml_diff>
--- a/wise-analysis/Wise-Financial-Model.xlsx
+++ b/wise-analysis/Wise-Financial-Model.xlsx
@@ -8,6 +8,8 @@
     <sheet state="visible" name="Assumptions" sheetId="3" r:id="rId7"/>
     <sheet state="visible" name="DCF" sheetId="4" r:id="rId8"/>
     <sheet state="visible" name="WACC" sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="Comparable Companies" sheetId="6" r:id="rId10"/>
+    <sheet state="visible" name="Valuation Summary" sheetId="7" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -115,70 +117,175 @@
 </comments>
 </file>
 
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment authorId="0" ref="B23">
+      <text>
+        <t xml:space="preserve">5,030.6 + 27,802.2 - 334.7 =32,498.1
+**numbers taking from 2026 Historical Financials</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="B22">
+      <text>
+        <t xml:space="preserve">wise revenue * median peer EV/R</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment authorId="0" ref="C3">
+      <text>
+        <t xml:space="preserve">EV/Revenue implied share value
+= 32,498 ÷ 1,024
+≈ $31.74</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="C2">
+      <text>
+        <t xml:space="preserve">Discounted cash flow (DCF) implied share value
+= 4620÷ 1,024
+≈ $4.51</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="C1">
+      <text>
+        <t xml:space="preserve">For the share-value calculation, your current market data implies roughly 1.024bn shares based on the $11.62bn market cap and $11.35 share price.</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="C4">
+      <text>
+        <t xml:space="preserve">P/E implied share value
+= 7,211 ÷ 1,024
+≈ $7.04</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="249">
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Ratio / Metric</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>FY2024</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>FY2025</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Driver</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>FY2026</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>FY2027 - F</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>FY2028 - F</t>
+  </si>
+  <si>
+    <t>FY2029 - F</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>Revenue Growth</t>
+  </si>
+  <si>
+    <t>Financial Metric</t>
+  </si>
   <si>
     <t>Metric</t>
   </si>
   <si>
-    <t>Ratio / Metric</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Driver</t>
-  </si>
-  <si>
-    <t>FY2024</t>
+    <t>Historical observation</t>
+  </si>
+  <si>
+    <t>FY2023 - A</t>
+  </si>
+  <si>
+    <t>Forecast assumption</t>
+  </si>
+  <si>
+    <t>FY2024 - A</t>
+  </si>
+  <si>
+    <t>FY2025 - A</t>
+  </si>
+  <si>
+    <t>Reason</t>
+  </si>
+  <si>
+    <t>FY2026 - A</t>
   </si>
   <si>
     <t>2027F</t>
   </si>
   <si>
-    <t>FY2025</t>
-  </si>
-  <si>
-    <t>B</t>
+    <t>Customer growth</t>
   </si>
   <si>
     <t>2028F</t>
   </si>
   <si>
-    <t>FY2026</t>
+    <t>Strong growth in customers</t>
+  </si>
+  <si>
+    <t>Net Revenue</t>
   </si>
   <si>
     <t>2029F</t>
   </si>
   <si>
-    <t>FY2027 - F</t>
-  </si>
-  <si>
-    <t>FY2028 - F</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
     <t>DCF Formula / Assumption</t>
   </si>
   <si>
-    <t>FY2029 - F</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>Revenue Growth</t>
-  </si>
-  <si>
-    <t>Historical observation</t>
+    <t>Continued geographic expansion</t>
+  </si>
+  <si>
+    <t>Transaction volume</t>
   </si>
   <si>
     <t>Formula</t>
   </si>
   <si>
-    <t>E</t>
+    <t>Increasing as customers grow</t>
   </si>
   <si>
     <t>Plain English</t>
@@ -187,67 +294,76 @@
     <t>Assumption</t>
   </si>
   <si>
-    <t>Forecast assumption</t>
+    <t>Higher customer usage</t>
   </si>
   <si>
     <t>Value</t>
   </si>
   <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>Reason</t>
+    <t>Geographic expansion</t>
+  </si>
+  <si>
+    <t>Increasing</t>
   </si>
   <si>
     <t>Explanation</t>
   </si>
   <si>
-    <t>G</t>
+    <t>continued exspansion</t>
+  </si>
+  <si>
+    <t>Wise adding markets and licences</t>
   </si>
   <si>
     <t>Revenue</t>
   </si>
   <si>
-    <t>Customer growth</t>
-  </si>
-  <si>
-    <t>H</t>
-  </si>
-  <si>
-    <t>Strong growth in customers</t>
-  </si>
-  <si>
-    <t>Financial Metric</t>
-  </si>
-  <si>
-    <t>Continued geographic expansion</t>
-  </si>
-  <si>
-    <t>FY2023 - A</t>
-  </si>
-  <si>
-    <t>Transaction volume</t>
-  </si>
-  <si>
-    <t>Increasing as customers grow</t>
-  </si>
-  <si>
-    <t>FY2024 - A</t>
-  </si>
-  <si>
-    <t>FY2025 - A</t>
-  </si>
-  <si>
-    <t>Higher customer usage</t>
-  </si>
-  <si>
-    <t>FY2026 - A</t>
+    <t>Product usage</t>
+  </si>
+  <si>
+    <t>Customers are using Wise for more everyday financial activity</t>
+  </si>
+  <si>
+    <t>Total Operating Expenses</t>
+  </si>
+  <si>
+    <t>Pricing</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> reduced prices over time - more competitive</t>
+  </si>
+  <si>
+    <t>gradual reduction</t>
+  </si>
+  <si>
+    <t>Lower prices can support customer and transaction growth</t>
+  </si>
+  <si>
+    <t>FY2027 Scenario</t>
+  </si>
+  <si>
+    <t>Operating Income</t>
+  </si>
+  <si>
+    <t>Bear</t>
+  </si>
+  <si>
+    <t>Base</t>
+  </si>
+  <si>
+    <t>Bull</t>
+  </si>
+  <si>
+    <t>Operating Profit Growth</t>
+  </si>
+  <si>
+    <t>Income Before Tax</t>
   </si>
   <si>
     <t>Previous Revenue × (1 + Growth)</t>
   </si>
   <si>
-    <t>Geographic expansion</t>
+    <t>Operating Margin</t>
   </si>
   <si>
     <t>Grows revenue using the assumed growth rate</t>
@@ -256,52 +372,43 @@
     <t>FY2027F Revenue Growth</t>
   </si>
   <si>
-    <t>Increasing</t>
-  </si>
-  <si>
-    <t>continued exspansion</t>
+    <t>Operating Profit</t>
   </si>
   <si>
     <t>Wise guidance midpoint</t>
   </si>
   <si>
-    <t>Wise adding markets and licences</t>
-  </si>
-  <si>
-    <t>Product usage</t>
-  </si>
-  <si>
-    <t>Net Revenue</t>
+    <t>Net Income</t>
+  </si>
+  <si>
+    <t>Net Income*</t>
   </si>
   <si>
     <t>EBIT (Operating income)</t>
   </si>
   <si>
-    <t>Customers are using Wise for more everyday financial activity</t>
-  </si>
-  <si>
-    <t>Operating Profit Growth</t>
-  </si>
-  <si>
-    <t>Pricing</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> reduced prices over time - more competitive</t>
-  </si>
-  <si>
-    <t>gradual reduction</t>
-  </si>
-  <si>
-    <t>Lower prices can support customer and transaction growth</t>
+    <t>Capex</t>
+  </si>
+  <si>
+    <t>Net Income Growth</t>
+  </si>
+  <si>
+    <t>Total Assets</t>
+  </si>
+  <si>
+    <t>Free Cash Flow*</t>
+  </si>
+  <si>
+    <t>Cash &amp; Cash Equivalents</t>
+  </si>
+  <si>
+    <t>Revenue growth</t>
   </si>
   <si>
     <t>EBIT</t>
   </si>
   <si>
-    <t>Operating Income</t>
-  </si>
-  <si>
-    <t>FY2027 Scenario</t>
+    <t>Total Debt</t>
   </si>
   <si>
     <t>Operating profit before interest and tax</t>
@@ -310,25 +417,31 @@
     <t>FY2028F Revenue Growth</t>
   </si>
   <si>
-    <t>Bear</t>
+    <t>Income before tax margin</t>
   </si>
   <si>
     <t>Model assumption</t>
   </si>
   <si>
-    <t>Base</t>
-  </si>
-  <si>
-    <t>Bull</t>
+    <t>Free Cash Flow Growth</t>
+  </si>
+  <si>
+    <t>Total Liabilities</t>
   </si>
   <si>
     <t>Tax</t>
   </si>
   <si>
-    <t>Net Income Growth</t>
-  </si>
-  <si>
-    <t>Operating Margin</t>
+    <t>Effective tax rate</t>
+  </si>
+  <si>
+    <t>Shareholders' Equity</t>
+  </si>
+  <si>
+    <t>Operating Cash Flow</t>
+  </si>
+  <si>
+    <t>Capex as % revenue</t>
   </si>
   <si>
     <t>EBIT × 24.49%</t>
@@ -337,48 +450,48 @@
     <t>Estimated tax on operating profit</t>
   </si>
   <si>
+    <t>Capital Expenditure</t>
+  </si>
+  <si>
+    <t>Depreciation and Ammortisation</t>
+  </si>
+  <si>
+    <t>D&amp;A as % revenue</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
     <t>FY2029F Revenue Growth</t>
   </si>
   <si>
-    <t>Operating Profit</t>
+    <t>Free Cash Flow</t>
   </si>
   <si>
     <t>NOPAT</t>
   </si>
   <si>
-    <t>Net Income*</t>
-  </si>
-  <si>
-    <t>Total Operating Expenses</t>
+    <t>FCF as % revenue</t>
+  </si>
+  <si>
+    <t>Net Profit Margin</t>
   </si>
   <si>
     <t>EBIT − Tax</t>
   </si>
   <si>
-    <t>Capex</t>
-  </si>
-  <si>
     <t>Operating profit after tax</t>
   </si>
   <si>
     <t>Tax Rate</t>
   </si>
   <si>
-    <t>Free Cash Flow Growth</t>
-  </si>
-  <si>
     <t>Based on FY2026 actual</t>
   </si>
   <si>
     <t>Depreciation</t>
   </si>
   <si>
-    <t>Free Cash Flow*</t>
-  </si>
-  <si>
-    <t>Revenue growth</t>
-  </si>
-  <si>
     <t>D&amp;A</t>
   </si>
   <si>
@@ -391,12 +504,6 @@
     <t>D&amp;A / Revenue</t>
   </si>
   <si>
-    <t>Income Before Tax</t>
-  </si>
-  <si>
-    <t>Income before tax margin</t>
-  </si>
-  <si>
     <t>Revenue × Capex %</t>
   </si>
   <si>
@@ -406,43 +513,67 @@
     <t>Working Capital / Revenue</t>
   </si>
   <si>
-    <t>Net Profit Margin</t>
-  </si>
-  <si>
-    <t>Effective tax rate</t>
-  </si>
-  <si>
     <t>Change in Working Capital</t>
   </si>
   <si>
-    <t>Net Income</t>
-  </si>
-  <si>
-    <t>Capex as % revenue</t>
+    <t>WACC Inputs</t>
+  </si>
+  <si>
+    <t>Terms</t>
+  </si>
+  <si>
+    <t>Definitions</t>
+  </si>
+  <si>
+    <t>CAPM Input</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Terminal Growth ↓ / WACC →</t>
   </si>
   <si>
     <t>Working Capital</t>
   </si>
   <si>
+    <t>8%</t>
+  </si>
+  <si>
     <t>Revenue × 1%</t>
   </si>
   <si>
+    <t>9%</t>
+  </si>
+  <si>
     <t>Estimated cash tied up in working capital</t>
   </si>
   <si>
+    <t>10%</t>
+  </si>
+  <si>
+    <t>11%</t>
+  </si>
+  <si>
     <t>Illustrative WACC assumption</t>
   </si>
   <si>
+    <t>12%</t>
+  </si>
+  <si>
+    <t>Market Value of Equity</t>
+  </si>
+  <si>
     <t>Temporary</t>
   </si>
   <si>
-    <t>Free Cash Flow</t>
-  </si>
-  <si>
-    <t>Total Assets</t>
-  </si>
-  <si>
-    <t>D&amp;A as % revenue</t>
+    <t>Share Price × Shares Outstanding</t>
+  </si>
+  <si>
+    <t>Risk-Free Rate</t>
+  </si>
+  <si>
+    <t>UK government bond</t>
   </si>
   <si>
     <t>FCF</t>
@@ -454,22 +585,40 @@
     <t>Cash generated after operating costs, tax and investment</t>
   </si>
   <si>
-    <t>FCF as % revenue</t>
-  </si>
-  <si>
     <t>Calculated WACC for Wise</t>
   </si>
   <si>
-    <t>Cash &amp; Cash Equivalents</t>
-  </si>
-  <si>
     <t>Wise info + assumptions</t>
   </si>
   <si>
+    <t>Wise</t>
+  </si>
+  <si>
     <t>Discount Factor (Wise's WACC)</t>
   </si>
   <si>
-    <t>Total Debt</t>
+    <t>Remitly</t>
+  </si>
+  <si>
+    <t>Adyen</t>
+  </si>
+  <si>
+    <t>PayPal</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Why it is comparable</t>
+  </si>
+  <si>
+    <t>Market Cap</t>
+  </si>
+  <si>
+    <t>Target; cross-border payments, multi-currency accounts and international money management</t>
+  </si>
+  <si>
+    <t>Enterprise Value</t>
   </si>
   <si>
     <t xml:space="preserve">Enterprise Value </t>
@@ -481,93 +630,132 @@
     <t>The total cost to buy an entire company, shows the real price tag of business operations</t>
   </si>
   <si>
+    <t>Closest peer for digital cross-border money transfers and consumer remittances</t>
+  </si>
+  <si>
     <t>Present Value</t>
   </si>
   <si>
-    <t>Total Liabilities</t>
+    <t>Global fintech/payment infrastructure with strong technology exposure and international operations</t>
+  </si>
+  <si>
+    <t>Method</t>
   </si>
   <si>
     <t>Sum of Present Value of Forecast FCF</t>
   </si>
   <si>
-    <t>Enterprise Value</t>
-  </si>
-  <si>
-    <t>Shareholders' Equity</t>
-  </si>
-  <si>
-    <t>Operating Cash Flow</t>
-  </si>
-  <si>
-    <t>Capital Expenditure</t>
-  </si>
-  <si>
-    <t>WACC Inputs</t>
-  </si>
-  <si>
-    <t>Terms</t>
-  </si>
-  <si>
-    <t>Definitions</t>
-  </si>
-  <si>
-    <t>Depreciation and Ammortisation</t>
-  </si>
-  <si>
-    <t>CAPM Input</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>Source</t>
-  </si>
-  <si>
-    <t>Terminal Growth ↓ / WACC →</t>
-  </si>
-  <si>
-    <t>8%</t>
-  </si>
-  <si>
-    <t>9%</t>
-  </si>
-  <si>
-    <t>10%</t>
-  </si>
-  <si>
-    <t>11%</t>
-  </si>
-  <si>
-    <t>12%</t>
-  </si>
-  <si>
-    <t>Market Value of Equity</t>
-  </si>
-  <si>
-    <t>Share Price × Shares Outstanding</t>
-  </si>
-  <si>
-    <t>Risk-Free Rate</t>
-  </si>
-  <si>
-    <t>UK government bond</t>
+    <t>~1,300</t>
+  </si>
+  <si>
+    <t>Equity Value ($m)</t>
+  </si>
+  <si>
+    <t>~6,100</t>
+  </si>
+  <si>
+    <t>Implied Share Value</t>
+  </si>
+  <si>
+    <t>Large-scale digital payments platform with consumer and merchant exposure</t>
+  </si>
+  <si>
+    <t>DCF</t>
+  </si>
+  <si>
+    <t>~$4.51</t>
+  </si>
+  <si>
+    <t>EV/Revenue</t>
+  </si>
+  <si>
+    <t>~$31.74</t>
+  </si>
+  <si>
+    <t>P/E</t>
+  </si>
+  <si>
+    <t>~$7.04</t>
+  </si>
+  <si>
+    <t>Comparable Median</t>
+  </si>
+  <si>
+    <t>~44%</t>
   </si>
   <si>
     <t>Debt</t>
   </si>
   <si>
+    <t>Term</t>
+  </si>
+  <si>
+    <t>[value]</t>
+  </si>
+  <si>
+    <t>Explanation + Formula</t>
+  </si>
+  <si>
     <t>Using FY2026 actual figure</t>
   </si>
   <si>
+    <t>EV / Revenue</t>
+  </si>
+  <si>
     <t>Wise Beta</t>
   </si>
   <si>
     <t>Documented market-data source</t>
   </si>
   <si>
+    <t>Enterprise Value =</t>
+  </si>
+  <si>
+    <t>Market Capitalisation + Debt - Cash</t>
+  </si>
+  <si>
+    <t>Shows how much investors are paying for each dollar of revenue generated; Enterprise Value ÷ Revenue</t>
+  </si>
+  <si>
+    <t>Price-to-Earnings (P/E) ratio</t>
+  </si>
+  <si>
+    <t>Tells you how much money investors are willing to pay for every single unit of a company's profit</t>
+  </si>
+  <si>
+    <t>Statistic</t>
+  </si>
+  <si>
+    <t>Company EV/R</t>
+  </si>
+  <si>
+    <t>Company P/E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P/E ratio = </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Market Capitalisation ÷ Net Income , e.g for Wise 11,620 ÷ 499 = 23.3x  </t>
+  </si>
+  <si>
+    <t>Minimum</t>
+  </si>
+  <si>
+    <t>Implied Equity Value (EV/R)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implied Enterprise Value  + Cash - Debt; this si the enterpirse value approach </t>
+  </si>
+  <si>
+    <t>Maximum</t>
+  </si>
+  <si>
     <t>Total Capital</t>
   </si>
   <si>
+    <t>Mean</t>
+  </si>
+  <si>
     <t>Equity + Debt, so x + 334.7</t>
   </si>
   <si>
@@ -577,7 +765,31 @@
     <t>Appropriate UK/GBP ERP source</t>
   </si>
   <si>
+    <t>Median</t>
+  </si>
+  <si>
+    <t>Wise revenue:</t>
+  </si>
+  <si>
+    <t>$2,502.80</t>
+  </si>
+  <si>
+    <t>Median peer EV/R:</t>
+  </si>
+  <si>
+    <t>Implied Enterprise Value</t>
+  </si>
+  <si>
+    <t>Implied Equity Value</t>
+  </si>
+  <si>
+    <t>Median peer P/E:</t>
+  </si>
+  <si>
     <t>Cost of Equity</t>
+  </si>
+  <si>
+    <t>Wise net income:</t>
   </si>
   <si>
     <t>Equity and debt weights</t>
@@ -716,6 +928,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.00x"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <sz val="10.0"/>
@@ -749,45 +965,42 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="31">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -795,16 +1008,15 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -818,7 +1030,32 @@
       <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="3" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -879,19 +1116,7 @@
       </border>
     </dxf>
   </dxfs>
-  <tableStyles count="14">
-    <tableStyle count="4" pivot="0" name="DCF-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
-    </tableStyle>
-    <tableStyle count="4" pivot="0" name="Assumptions-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
-    </tableStyle>
+  <tableStyles count="20">
     <tableStyle count="4" pivot="0" name="Historical Financials-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
@@ -904,7 +1129,13 @@
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
-    <tableStyle count="4" pivot="0" name="DCF-style 2">
+    <tableStyle count="4" pivot="0" name="Assumptions-style">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+    <tableStyle count="4" pivot="0" name="DCF-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -916,13 +1147,19 @@
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
-    <tableStyle count="4" pivot="0" name="DCF-style 3">
+    <tableStyle count="4" pivot="0" name="DCF-style 2">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
     <tableStyle count="4" pivot="0" name="Assumptions-style 3">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+    <tableStyle count="4" pivot="0" name="DCF-style 3">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -964,6 +1201,42 @@
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
+    <tableStyle count="4" pivot="0" name="Comparable Companies-style">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+    <tableStyle count="4" pivot="0" name="Comparable Companies-style 2">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+    <tableStyle count="4" pivot="0" name="Comparable Companies-style 3">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+    <tableStyle count="4" pivot="0" name="Comparable Companies-style 4">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+    <tableStyle count="4" pivot="0" name="Comparable Companies-style 5">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+    <tableStyle count="4" pivot="0" name="Valuation Summary-style">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
   </tableStyles>
 </styleSheet>
 </file>
@@ -988,12 +1261,20 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:H17" displayName="Table1" name="Table1" id="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:H17" displayName="Table1" name="Table1" id="1">
   <tableColumns count="8">
     <tableColumn name="A" id="1"/>
     <tableColumn name="B" id="2"/>
@@ -1063,8 +1344,64 @@
 </table>
 </file>
 
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E10" displayName="Table13" name="Table13" id="15">
+  <tableColumns count="5">
+    <tableColumn name="Metric" id="1"/>
+    <tableColumn name="Wise" id="2"/>
+    <tableColumn name="Remitly" id="3"/>
+    <tableColumn name="Adyen" id="4"/>
+    <tableColumn name="PayPal" id="5"/>
+  </tableColumns>
+  <tableStyleInfo name="Comparable Companies-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="G1:H5" displayName="Table12" name="Table12" id="16">
+  <tableColumns count="2">
+    <tableColumn name="Company" id="1"/>
+    <tableColumn name="Why it is comparable" id="2"/>
+  </tableColumns>
+  <tableStyleInfo name="Comparable Companies-style 2" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="G8:H14" displayName="Valuation_Calculation" name="Valuation_Calculation" id="17">
+  <tableColumns count="2">
+    <tableColumn name="Term" id="1"/>
+    <tableColumn name="Explanation + Formula" id="2"/>
+  </tableColumns>
+  <tableStyleInfo name="Comparable Companies-style 3" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A13:E17" displayName="Table14" name="Table14" id="18">
+  <tableColumns count="5">
+    <tableColumn name="Statistic" id="1"/>
+    <tableColumn name="EV / Revenue" id="2"/>
+    <tableColumn name="Company EV/R" id="3"/>
+    <tableColumn name="P/E" id="4"/>
+    <tableColumn name="Company P/E" id="5"/>
+  </tableColumns>
+  <tableStyleInfo name="Comparable Companies-style 4" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A20:B26" displayName="Table15" name="Table15" id="19">
+  <tableColumns count="2">
+    <tableColumn name="Wise revenue:" id="1"/>
+    <tableColumn name="$2,502.80" id="2"/>
+  </tableColumns>
+  <tableStyleInfo name="Comparable Companies-style 5" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:G8" displayName="Table2" name="Table2" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:G8" displayName="Table2" name="Table2" id="2">
   <tableColumns count="7">
     <tableColumn name="Ratio / Metric" id="1"/>
     <tableColumn name="FY2024" id="2"/>
@@ -1078,6 +1415,17 @@
 </table>
 </file>
 
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C5" displayName="Table16" name="Table16" id="20">
+  <tableColumns count="3">
+    <tableColumn name="Method" id="1"/>
+    <tableColumn name="Equity Value ($m)" id="2"/>
+    <tableColumn name="Implied Share Value" id="3"/>
+  </tableColumns>
+  <tableStyleInfo name="Valuation Summary-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:D6" displayName="Table3" name="Table3" id="3">
   <tableColumns count="4">
@@ -1091,7 +1439,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A8:D14" displayName="Table4" name="Table4" id="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A8:D14" displayName="Table4" name="Table4" id="5">
   <tableColumns count="4">
     <tableColumn name="FY2027 Scenario" id="1"/>
     <tableColumn name="Bear" id="2"/>
@@ -1103,7 +1451,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A16:D22" displayName="Table6" name="Table6" id="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A16:D22" displayName="Table6" name="Table6" id="7">
   <tableColumns count="4">
     <tableColumn name="Assumption" id="1"/>
     <tableColumn name="2027F" id="2"/>
@@ -1127,7 +1475,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="F1:H10" displayName="Table7" name="Table7" id="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="F1:H10" displayName="Table7" name="Table7" id="6">
   <tableColumns count="3">
     <tableColumn name="DCF Formula / Assumption" id="1"/>
     <tableColumn name="Formula" id="2"/>
@@ -1138,7 +1486,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="J1:L9" displayName="Table8" name="Table8" id="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="J1:L9" displayName="Table8" name="Table8" id="8">
   <tableColumns count="3">
     <tableColumn name="Assumption" id="1"/>
     <tableColumn name="Value" id="2"/>
@@ -1368,61 +1716,61 @@
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>7</v>
-      </c>
       <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" ht="22.5" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>15</v>
+      <c r="H2" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B3" s="12">
+        <v>30</v>
+      </c>
+      <c r="B3" s="6">
         <v>1020.4</v>
       </c>
       <c r="C3" s="4">
@@ -1449,33 +1797,33 @@
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B4" s="12">
+        <v>49</v>
+      </c>
+      <c r="B4" s="6">
         <v>580.1</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="6">
         <v>1126.0</v>
       </c>
-      <c r="D4" s="12">
+      <c r="D4" s="6">
         <v>1370.7</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="6">
         <v>1912.1</v>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="6">
         <v>2283.19</v>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="6">
         <v>2702.12</v>
       </c>
-      <c r="H4" s="12">
+      <c r="H4" s="6">
         <v>3170.13</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B5" s="4">
         <v>189.6</v>
@@ -1501,7 +1849,7 @@
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="B6" s="4">
         <v>176.7</v>
@@ -1530,7 +1878,7 @@
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>99</v>
+        <v>67</v>
       </c>
       <c r="B7" s="4">
         <v>137.5</v>
@@ -1556,47 +1904,47 @@
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="B8" s="12">
+        <v>72</v>
+      </c>
+      <c r="B8" s="6">
         <v>14695.7</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="6">
         <v>19022.5</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="6">
         <v>24781.1</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="6">
         <v>33259.8</v>
       </c>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="B9" s="12">
+        <v>74</v>
+      </c>
+      <c r="B9" s="6">
         <v>9480.2</v>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="6">
         <v>13245.7</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="6">
         <v>18066.3</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="6">
         <v>27802.2</v>
       </c>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>117</v>
+        <v>77</v>
       </c>
       <c r="B10" s="4">
         <v>326.4</v>
@@ -1616,73 +1964,73 @@
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="B11" s="12">
+        <v>83</v>
+      </c>
+      <c r="B11" s="6">
         <v>13983.6</v>
       </c>
-      <c r="C11" s="12">
+      <c r="C11" s="6">
         <v>17857.4</v>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="6">
         <v>23043.7</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="6">
         <v>31334.6</v>
       </c>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="B12" s="12">
+        <v>86</v>
+      </c>
+      <c r="B12" s="6">
         <v>712.2</v>
       </c>
-      <c r="C12" s="12">
+      <c r="C12" s="6">
         <v>1165.1</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="6">
         <v>1737.4</v>
       </c>
-      <c r="E12" s="12">
+      <c r="E12" s="6">
         <v>1925.2</v>
       </c>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="B13" s="12">
+        <v>87</v>
+      </c>
+      <c r="B13" s="6">
         <v>4727.4</v>
       </c>
-      <c r="C13" s="12">
+      <c r="C13" s="6">
         <v>4075.1</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="6">
         <v>5719.5</v>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="6">
         <v>7553.9</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="6">
         <v>857.1</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="6">
         <v>1033.2</v>
       </c>
-      <c r="H13" s="12">
+      <c r="H13" s="6">
         <v>1237.3</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>127</v>
+        <v>91</v>
       </c>
       <c r="B14" s="4">
         <v>10.6</v>
@@ -1708,10 +2056,10 @@
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>131</v>
+        <v>92</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>133</v>
+        <v>94</v>
       </c>
       <c r="C15" s="4">
         <v>14.3</v>
@@ -1728,7 +2076,7 @@
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B16" s="4">
         <v>188.1</v>
@@ -1748,7 +2096,7 @@
       <c r="G16" s="4">
         <v>998.0</v>
       </c>
-      <c r="H16" s="12">
+      <c r="H16" s="6">
         <v>1197.4</v>
       </c>
     </row>
@@ -1789,10 +2137,10 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>9</v>
@@ -1801,17 +2149,17 @@
         <v>11</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" s="9">
+        <v>16</v>
+      </c>
+      <c r="B2" s="8">
         <f>'Historical Financials'!C3/'Historical Financials'!B3-1</f>
         <v>0.7405919247</v>
       </c>
@@ -1823,19 +2171,19 @@
         <f>('Historical Financials'!E3-'Historical Financials'!D3)/'Historical Financials'!D3</f>
         <v>0.1924341322</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="8">
         <v>0.175</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="8">
         <v>0.17</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="8">
         <v>0.16</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B3" s="10">
         <f>'Historical Financials'!C5/'Historical Financials'!B5-1</f>
@@ -1855,7 +2203,7 @@
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B4" s="10">
         <f>'Historical Financials'!C7/'Historical Financials'!B7-1</f>
@@ -1895,7 +2243,7 @@
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="B6" s="10">
         <f>'Historical Financials'!C5/'Historical Financials'!C3</f>
@@ -1915,7 +2263,7 @@
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B7" s="10">
         <f>'Historical Financials'!C7/'Historical Financials'!C3</f>
@@ -1969,134 +2317,134 @@
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>26</v>
+      <c r="A1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="6">
+        <v>29</v>
+      </c>
+      <c r="C2" s="7">
         <v>0.15</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C3" s="6">
+      <c r="C3" s="7">
         <v>0.18</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C8" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D8" s="9" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="13">
+        <v>46</v>
+      </c>
+      <c r="B9" s="12">
         <v>2703.02</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="12">
         <v>2878.22</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="12">
         <v>3053.42</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B10" s="14">
+        <v>62</v>
+      </c>
+      <c r="B10" s="13">
         <v>0.15</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="13">
         <v>0.2</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="13">
         <v>0.24</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="B11" s="15">
         <v>405.45</v>
@@ -2110,7 +2458,7 @@
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B12" s="15">
         <v>305.35</v>
@@ -2124,7 +2472,7 @@
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="B13" s="15">
         <v>189.21</v>
@@ -2138,7 +2486,7 @@
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="B14" s="15">
         <v>667.89</v>
@@ -2151,100 +2499,100 @@
       </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
-      <c r="A16" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>10</v>
+      <c r="A16" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="B17" s="11">
+        <v>75</v>
+      </c>
+      <c r="B17" s="14">
         <v>0.175</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="8">
         <v>0.17</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="14">
         <v>0.16</v>
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="B18" s="11">
+        <v>80</v>
+      </c>
+      <c r="B18" s="14">
         <v>0.25</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="8">
         <v>0.24</v>
       </c>
-      <c r="D18" s="11">
+      <c r="D18" s="14">
         <v>0.23</v>
       </c>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B19" s="11">
+        <v>85</v>
+      </c>
+      <c r="B19" s="14">
         <v>0.2449</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="8">
         <v>0.2449</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="14">
         <v>0.2449</v>
       </c>
     </row>
     <row r="20" ht="22.5" customHeight="1">
       <c r="A20" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B20" s="11">
+        <v>88</v>
+      </c>
+      <c r="B20" s="14">
         <v>0.01</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="8">
         <v>0.01</v>
       </c>
-      <c r="D20" s="11">
+      <c r="D20" s="14">
         <v>0.01</v>
       </c>
     </row>
     <row r="21" ht="22.5" customHeight="1">
       <c r="A21" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="B21" s="11">
+        <v>93</v>
+      </c>
+      <c r="B21" s="14">
         <v>0.00575</v>
       </c>
-      <c r="C21" s="9">
+      <c r="C21" s="8">
         <v>0.0058</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="14">
         <v>0.00575</v>
       </c>
     </row>
     <row r="22" ht="22.5" customHeight="1">
       <c r="A22" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="B22" s="11">
+        <v>98</v>
+      </c>
+      <c r="B22" s="14">
         <v>0.28</v>
       </c>
-      <c r="C22" s="9">
+      <c r="C22" s="8">
         <v>0.29</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="14">
         <v>0.3</v>
       </c>
     </row>
@@ -2281,287 +2629,287 @@
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>27</v>
+      <c r="A1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B2" s="8">
+        <v>46</v>
+      </c>
+      <c r="B2" s="11">
         <f>'Historical Financials'!F3</f>
         <v>2940.79</v>
       </c>
-      <c r="C2" s="8">
+      <c r="C2" s="11">
         <f>'Historical Financials'!G3</f>
         <v>3440.7243</v>
       </c>
-      <c r="D2" s="8">
+      <c r="D2" s="11">
         <f>'Historical Financials'!H3</f>
         <v>3991.240188</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="K2" s="11">
+        <v>64</v>
+      </c>
+      <c r="K2" s="14">
         <v>0.175</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B3" s="8">
+        <v>69</v>
+      </c>
+      <c r="B3" s="11">
         <f>'Historical Financials'!F5</f>
         <v>657.6</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="11">
         <f>'Historical Financials'!G5</f>
         <v>738.62</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="11">
         <f>'Historical Financials'!H5</f>
         <v>821.1</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="K3" s="11">
+        <v>79</v>
+      </c>
+      <c r="K3" s="14">
         <v>0.17</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B4" s="8">
+        <v>84</v>
+      </c>
+      <c r="B4" s="11">
         <f>B3*Assumptions!B19</f>
         <v>161.04624</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="11">
         <f>C3*Assumptions!C19</f>
         <v>180.888038</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="11">
         <f>D3*Assumptions!D19</f>
         <v>201.08739</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="K4" s="11">
+        <v>95</v>
+      </c>
+      <c r="K4" s="14">
         <v>0.16</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B5" s="8">
+        <v>97</v>
+      </c>
+      <c r="B5" s="11">
         <f t="shared" ref="B5:D5" si="1">B3-B4</f>
         <v>496.55376</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="11">
         <f t="shared" si="1"/>
         <v>557.731962</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="11">
         <f t="shared" si="1"/>
         <v>620.01261</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>78</v>
+        <v>100</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="K5" s="11">
+        <v>102</v>
+      </c>
+      <c r="K5" s="14">
         <v>0.2449</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="B6" s="8">
+        <v>104</v>
+      </c>
+      <c r="B6" s="11">
         <f>'Historical Financials'!F3 * Assumptions!B21</f>
         <v>16.9095425</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="11">
         <f>'Historical Financials'!G3 * Assumptions!C21</f>
         <v>19.95620094</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="11">
         <f>'Historical Financials'!H3 * Assumptions!D21</f>
         <v>22.94963108</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="K6" s="11">
+        <v>108</v>
+      </c>
+      <c r="K6" s="14">
         <v>0.00575</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B7" s="8">
+        <v>70</v>
+      </c>
+      <c r="B7" s="11">
         <f>'Historical Financials'!F14</f>
         <v>29.41</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="11">
         <f>'Historical Financials'!G14</f>
         <v>34.41</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="11">
         <f>'Historical Financials'!H14</f>
         <v>39.91</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="K7" s="11">
+        <v>111</v>
+      </c>
+      <c r="K7" s="14">
         <v>0.01</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B8" s="8">
+        <v>112</v>
+      </c>
+      <c r="B8" s="11">
         <f t="shared" ref="B8:D8" si="2">B2*0.01</f>
         <v>29.4079</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="11">
         <f t="shared" si="2"/>
         <v>34.407243</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="11">
         <f t="shared" si="2"/>
         <v>39.91240188</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>101</v>
+        <v>119</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>103</v>
+        <v>123</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="K8" s="11">
+        <v>126</v>
+      </c>
+      <c r="K8" s="14">
         <v>0.1</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>105</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="B9" s="8">
+        <v>96</v>
+      </c>
+      <c r="B9" s="11">
         <f t="shared" ref="B9:D9" si="3">B5+B6-B7-B8</f>
         <v>454.6454025</v>
       </c>
@@ -2569,86 +2917,86 @@
         <f t="shared" si="3"/>
         <v>508.8709199</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="11">
         <f t="shared" si="3"/>
         <v>563.1398392</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>109</v>
+        <v>133</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>110</v>
+        <v>134</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>111</v>
+        <v>135</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="K9" s="11">
+        <v>136</v>
+      </c>
+      <c r="K9" s="14">
         <v>0.1204</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="B10" s="8">
+        <v>139</v>
+      </c>
+      <c r="B10" s="11">
         <f>ROUND(1/(1+12.04%)^1,4)</f>
         <v>0.8925</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="11">
         <f>ROUND(1/(1+12.04%)^2,4)</f>
         <v>0.7966</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="11">
         <f>ROUND(1/(1+12.04%)^3,4)</f>
         <v>0.711</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>119</v>
+        <v>149</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B11" s="8">
+        <v>152</v>
+      </c>
+      <c r="B11" s="11">
         <f t="shared" ref="B11:D11" si="4">ROUND((B9*B10),3)</f>
         <v>405.771</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="11">
         <f t="shared" si="4"/>
         <v>405.367</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="11">
         <f t="shared" si="4"/>
         <v>400.392</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="s">
-        <v>123</v>
-      </c>
-      <c r="C13" s="18">
+      <c r="A13" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="C13" s="23">
         <f>SUM(B11:D11)</f>
         <v>1211.53</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="C14" s="18">
+      <c r="A14" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="C14" s="23">
         <f>C13+WACC!I14</f>
         <v>4620.412</v>
       </c>
@@ -2688,341 +3036,341 @@
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="N1" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="O1" s="19" t="s">
-        <v>137</v>
-      </c>
-      <c r="P1" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="Q1" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="R1" s="19" t="s">
-        <v>140</v>
+      <c r="A1" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="N1" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="O1" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="P1" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="Q1" s="17" t="s">
+        <v>125</v>
+      </c>
+      <c r="R1" s="17" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="B2" s="20">
+        <v>128</v>
+      </c>
+      <c r="B2" s="18">
         <v>8920.0</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>142</v>
+        <v>128</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="I2" s="21">
+        <v>131</v>
+      </c>
+      <c r="I2" s="19">
         <v>0.052392</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="M2" s="11">
+        <v>132</v>
+      </c>
+      <c r="M2" s="14">
         <v>0.015</v>
       </c>
-      <c r="N2" s="22">
+      <c r="N2" s="20">
         <f>ROUND(454.65/(1+8%)+508.72/(1+8%)^2+563.18/(1+8%)^3+((446.238*(1+1.5%))/(8%-1.5%))/(1+8%)^3,3)</f>
         <v>6835.752</v>
       </c>
-      <c r="O2" s="22">
+      <c r="O2" s="20">
         <f>ROUND(454.65/(1+9%)+508.72/(1+9%)^2+563.18/(1+9%)^3+((446.238*(1+1.5%))/(9%-1.5%))/(1+9%)^3,3)</f>
         <v>5943.452</v>
       </c>
-      <c r="P2" s="22">
+      <c r="P2" s="20">
         <f>ROUND(454.65/(1+10%)+508.72/(1+10%)^2+563.18/(1+10%)^3+((446.238*(1+1.5%))/(10%-1.5%))/(1+10%)^3,3)</f>
         <v>5260.334</v>
       </c>
-      <c r="Q2" s="22">
+      <c r="Q2" s="20">
         <f>ROUND(454.65/(1+11%)+508.72/(1+11%)^2+563.18/(1+11%)^3+((446.238*(1+1.5%))/(11%-1.5%))/(1+11%)^3,3)</f>
         <v>4720.377</v>
       </c>
-      <c r="R2" s="22">
+      <c r="R2" s="20">
         <f>ROUND(454.65/(1+12%)+508.72/(1+12%)^2+563.18/(1+12%)^3+((446.238*(1+1.5%))/(12%-1.5%))/(1+12%)^3,3)</f>
         <v>4282.706</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="B3" s="4">
         <v>334.7</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>146</v>
+        <v>169</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>173</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>147</v>
+        <v>175</v>
       </c>
       <c r="I3" s="15">
         <v>1.4113</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="M3" s="11">
+        <v>176</v>
+      </c>
+      <c r="M3" s="14">
         <v>0.02</v>
       </c>
-      <c r="N3" s="22">
+      <c r="N3" s="20">
         <f>ROUND(454.65/(1+8%)+508.72/(1+8%)^2+563.18/(1+8%)^3+((446.238*(1+2%))/(8%-2%))/(1+8%)^3,3)</f>
         <v>7326.236</v>
       </c>
-      <c r="O3" s="22">
+      <c r="O3" s="20">
         <f>ROUND(454.65/(1+9%)+508.72/(1+9%)^2+563.18/(1+9%)^3+((446.238*(1+2%))/(9%-2%))/(1+9%)^3,3)</f>
         <v>6301.156</v>
       </c>
-      <c r="P3" s="22">
+      <c r="P3" s="20">
         <f>ROUND(454.65/(1+10%)+508.72/(1+10%)^2+563.18/(1+10%)^3+((446.238*(1+2%))/(10%-2%))/(1+10%)^3,3)</f>
         <v>5531.505</v>
       </c>
-      <c r="Q3" s="22">
+      <c r="Q3" s="20">
         <f>ROUND(454.65/(1+11%)+508.72/(1+11%)^2+563.18/(1+11%)^3+((446.238*(1+2%))/(11%-2%))/(1+11%)^3,3)</f>
         <v>4932.176</v>
       </c>
-      <c r="R3" s="22">
+      <c r="R3" s="20">
         <f>ROUND(454.65/(1+12%)+508.72/(1+12%)^2+563.18/(1+12%)^3+((446.238*(1+2%))/(12%-2%))/(1+12%)^3,3)</f>
         <v>4452.105</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="B4" s="23">
+        <v>191</v>
+      </c>
+      <c r="B4" s="25">
         <f>SUM(B2:B3)</f>
         <v>9254.7</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>150</v>
+        <v>191</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>193</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="I4" s="21">
+        <v>194</v>
+      </c>
+      <c r="I4" s="19">
         <v>0.0503</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="M4" s="11">
+        <v>195</v>
+      </c>
+      <c r="M4" s="14">
         <v>0.025</v>
       </c>
-      <c r="N4" s="22">
+      <c r="N4" s="20">
         <f>ROUND(454.65/(1+8%)+508.72/(1+8%)^2+563.18/(1+8%)^3+((446.238*(1+2.5%))/(8%-2.5%))/(1+8%)^3,3)</f>
         <v>7905.898</v>
       </c>
-      <c r="O4" s="22">
+      <c r="O4" s="20">
         <f>ROUND(454.65/(1+9%)+508.72/(1+9%)^2+563.18/(1+9%)^3+((446.238*(1+2.5%))/(9%-2.5%))/(1+9%)^3,3)</f>
         <v>6713.892</v>
       </c>
-      <c r="P4" s="22">
+      <c r="P4" s="20">
         <f>ROUND(454.65/(1+10%)+508.72/(1+10%)^2+563.18/(1+10%)^3+((446.238*(1+2.5%))/(10%-2.5%))/(1+10%)^3,3)</f>
         <v>5838.831</v>
       </c>
-      <c r="Q4" s="22">
+      <c r="Q4" s="20">
         <f>ROUND(454.65/(1+11%)+508.72/(1+11%)^2+563.18/(1+11%)^3+((446.238*(1+2.5%))/(11%-2.5%))/(1+11%)^3,3)</f>
         <v>5168.893</v>
       </c>
-      <c r="R4" s="22">
+      <c r="R4" s="20">
         <f>ROUND(454.65/(1+12%)+508.72/(1+12%)^2+563.18/(1+12%)^3+((446.238*(1+2.5%))/(12%-2.5%))/(1+12%)^3,3)</f>
         <v>4639.336</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="B5" s="21">
+        <v>203</v>
+      </c>
+      <c r="B5" s="19">
         <v>0.1234</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="I5" s="21">
+        <v>205</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="I5" s="19">
         <f>I2+(I3*I4)</f>
         <v>0.12338039</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="M5" s="11">
+        <v>207</v>
+      </c>
+      <c r="M5" s="14">
         <v>0.03</v>
       </c>
-      <c r="N5" s="22">
+      <c r="N5" s="20">
         <f>ROUND(454.65/(1+8%)+508.72/(1+8%)^2+563.18/(1+8%)^3+((446.238*(1+3%))/(8%-3%))/(1+8%)^3,3)</f>
         <v>8601.493</v>
       </c>
-      <c r="O5" s="22">
+      <c r="O5" s="20">
         <f>ROUND(454.65/(1+9%)+508.72/(1+9%)^2+563.18/(1+9%)^3+((446.238*(1+3%))/(9%-3%))/(1+9%)^3,3)</f>
         <v>7195.417</v>
       </c>
-      <c r="P5" s="22">
+      <c r="P5" s="20">
         <f>ROUND(454.65/(1+10%)+508.72/(1+10%)^2+563.18/(1+10%)^3+((446.238*(1+3%))/(10%-3%))/(1+10%)^3,3)</f>
         <v>6190.062</v>
       </c>
-      <c r="Q5" s="22">
+      <c r="Q5" s="20">
         <f>ROUND(454.65/(1+11%)+508.72/(1+11%)^2+563.18/(1+11%)^3+((446.238*(1+3%))/(11%-3%))/(1+11%)^3,3)</f>
         <v>5435.2</v>
       </c>
-      <c r="R5" s="22">
+      <c r="R5" s="20">
         <f>ROUND(454.65/(1+12%)+508.72/(1+12%)^2+563.18/(1+12%)^3+((446.238*(1+3%))/(12%-3%))/(1+12%)^3,3)</f>
         <v>4847.37</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="B6" s="11">
+        <v>208</v>
+      </c>
+      <c r="B6" s="14">
         <v>0.0535</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="M6" s="11">
+        <v>209</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="M6" s="14">
         <v>0.035</v>
       </c>
-      <c r="N6" s="22">
+      <c r="N6" s="20">
         <f>ROUND(454.65/(1+8%)+508.72/(1+8%)^2+563.18/(1+8%)^3+((446.238*(1+3.5%))/(8%-3.5%))/(1+8%)^3,3)</f>
         <v>9451.665</v>
       </c>
-      <c r="O6" s="22">
+      <c r="O6" s="20">
         <f>ROUND(454.65/(1+9%)+508.72/(1+9%)^2+563.18/(1+9%)^3+((446.238*(1+3.5%))/(9%-3.5%))/(1+9%)^3,3)</f>
         <v>7764.492</v>
       </c>
-      <c r="P6" s="22">
+      <c r="P6" s="20">
         <f>ROUND(454.65/(1+10%)+508.72/(1+10%)^2+563.18/(1+10%)^3+((446.238*(1+3.5%))/(10%-3.5%))/(1+10%)^3,3)</f>
         <v>6595.327</v>
       </c>
-      <c r="Q6" s="22">
+      <c r="Q6" s="20">
         <f>ROUND(454.65/(1+11%)+508.72/(1+11%)^2+563.18/(1+11%)^3+((446.238*(1+3.5%))/(11%-3.5%))/(1+11%)^3,3)</f>
         <v>5737.014</v>
       </c>
-      <c r="R6" s="22">
+      <c r="R6" s="20">
         <f>ROUND(454.65/(1+12%)+508.72/(1+12%)^2+563.18/(1+12%)^3+((446.238*(1+3.5%))/(12%-3.5%))/(1+12%)^3,3)</f>
         <v>5079.878</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="B7" s="11">
+        <v>102</v>
+      </c>
+      <c r="B7" s="14">
         <v>0.2449</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>160</v>
+        <v>211</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>161</v>
+        <v>212</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="B8" s="22">
+        <v>213</v>
+      </c>
+      <c r="B8" s="20">
         <f>ROUND(B2/B4,4)</f>
         <v>0.9638</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>163</v>
+        <v>214</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>24</v>
+        <v>215</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="B9" s="22">
+        <v>216</v>
+      </c>
+      <c r="B9" s="20">
         <f>ROUND(B3/B4,4)</f>
         <v>0.0362</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>167</v>
+        <v>217</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>218</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>168</v>
+        <v>219</v>
       </c>
       <c r="I9" s="15">
         <v>563.18</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="B10" s="22">
+      <c r="A10" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B10" s="20">
         <f>ROUND((B8*B5)+(B9*B6*(1-B7)),4)</f>
         <v>0.1204</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>170</v>
+        <v>221</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>171</v>
+        <v>222</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>169</v>
+        <v>220</v>
       </c>
       <c r="I10" s="15">
         <v>0.1204</v>
@@ -3030,27 +3378,27 @@
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="E11" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>172</v>
+        <v>175</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>223</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="I11" s="21">
+        <v>224</v>
+      </c>
+      <c r="I11" s="19">
         <v>0.025</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="E12" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>174</v>
+        <v>208</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>225</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>175</v>
+        <v>226</v>
       </c>
       <c r="I12" s="15">
         <f>ROUND((I9*(1+I11))/I10-0.025,4)</f>
@@ -3059,13 +3407,13 @@
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="E13" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>177</v>
+        <v>227</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>228</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>178</v>
+        <v>229</v>
       </c>
       <c r="I13" s="15">
         <f>ROUND(1/(1+I10)^3,4)</f>
@@ -3074,13 +3422,13 @@
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="E14" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>179</v>
+        <v>226</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>230</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>180</v>
+        <v>231</v>
       </c>
       <c r="I14" s="15">
         <f>ROUND(I12*I13,3)</f>
@@ -3089,43 +3437,43 @@
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="E15" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>182</v>
+        <v>232</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="E16" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>183</v>
+        <v>224</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
-      <c r="E17" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="I17" s="5" t="s">
-        <v>186</v>
+      <c r="E17" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="I17" s="9" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
-      <c r="E18" s="7" t="s">
-        <v>187</v>
+      <c r="E18" s="3" t="s">
+        <v>238</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>188</v>
+        <v>239</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>189</v>
+        <v>240</v>
       </c>
       <c r="I18" s="15">
         <v>1211.52</v>
@@ -3133,13 +3481,13 @@
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="E19" s="4" t="s">
-        <v>190</v>
+        <v>241</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>191</v>
+        <v>242</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>180</v>
+        <v>231</v>
       </c>
       <c r="I19" s="15">
         <v>3408.882</v>
@@ -3147,13 +3495,13 @@
     </row>
     <row r="20" ht="22.5" customHeight="1">
       <c r="E20" s="4" t="s">
-        <v>192</v>
+        <v>243</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>193</v>
+        <v>244</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="I20" s="15">
         <v>4620.412</v>
@@ -3161,13 +3509,13 @@
     </row>
     <row r="21" ht="22.5" customHeight="1">
       <c r="E21" s="4" t="s">
-        <v>194</v>
+        <v>245</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>195</v>
+        <v>246</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>196</v>
+        <v>247</v>
       </c>
       <c r="I21" s="15">
         <v>27802.2</v>
@@ -3175,7 +3523,7 @@
     </row>
     <row r="22" ht="22.5" customHeight="1">
       <c r="H22" s="4" t="s">
-        <v>197</v>
+        <v>248</v>
       </c>
       <c r="I22" s="15">
         <v>334.7</v>
@@ -3183,7 +3531,7 @@
     </row>
     <row r="23" ht="22.5" customHeight="1">
       <c r="H23" s="4" t="s">
-        <v>190</v>
+        <v>241</v>
       </c>
       <c r="I23" s="15">
         <f>I20+I21-I22</f>
@@ -3207,4 +3555,497 @@
     <tablePart r:id="rId15"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="19.0"/>
+    <col customWidth="1" min="2" max="2" width="13.5"/>
+    <col customWidth="1" min="3" max="3" width="13.63"/>
+    <col customWidth="1" min="4" max="4" width="12.63"/>
+    <col customWidth="1" min="7" max="7" width="21.75"/>
+    <col customWidth="1" min="8" max="8" width="78.13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22.5" customHeight="1">
+      <c r="A1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" ht="22.5" customHeight="1">
+      <c r="A2" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B2" s="21">
+        <v>11620.0</v>
+      </c>
+      <c r="C2" s="21">
+        <v>4270.0</v>
+      </c>
+      <c r="D2" s="21">
+        <v>30950.0</v>
+      </c>
+      <c r="E2" s="21">
+        <v>44920.0</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="3" ht="22.5" customHeight="1">
+      <c r="A3" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B3" s="21">
+        <v>6720.0</v>
+      </c>
+      <c r="C3" s="21">
+        <v>3640.0</v>
+      </c>
+      <c r="D3" s="21">
+        <v>17290.0</v>
+      </c>
+      <c r="E3" s="21">
+        <v>47890.0</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="4" ht="22.5" customHeight="1">
+      <c r="A4" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="21">
+        <v>2503.0</v>
+      </c>
+      <c r="C4" s="21">
+        <v>1810.0</v>
+      </c>
+      <c r="D4" s="21">
+        <v>2950.0</v>
+      </c>
+      <c r="E4" s="21">
+        <v>34130.0</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="15">
+        <v>591.0</v>
+      </c>
+      <c r="C5" s="15">
+        <v>77.0</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="6" ht="22.5" customHeight="1">
+      <c r="A6" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" s="15">
+        <v>499.0</v>
+      </c>
+      <c r="C6" s="15">
+        <v>305.0</v>
+      </c>
+      <c r="D6" s="21">
+        <v>1130.0</v>
+      </c>
+      <c r="E6" s="21">
+        <v>4900.0</v>
+      </c>
+    </row>
+    <row r="7" ht="22.5" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="19">
+        <v>0.192</v>
+      </c>
+      <c r="C7" s="19">
+        <v>0.238</v>
+      </c>
+      <c r="D7" s="19">
+        <v>0.179</v>
+      </c>
+      <c r="E7" s="19">
+        <v>0.057</v>
+      </c>
+    </row>
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B8" s="19">
+        <v>0.236</v>
+      </c>
+      <c r="C8" s="19">
+        <v>0.043</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="E8" s="19">
+        <v>0.183</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="9" ht="22.5" customHeight="1">
+      <c r="A9" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B9" s="15">
+        <v>2.69</v>
+      </c>
+      <c r="C9" s="15">
+        <v>2.01</v>
+      </c>
+      <c r="D9" s="15">
+        <v>5.86</v>
+      </c>
+      <c r="E9" s="15">
+        <v>1.4</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="10" ht="22.5" customHeight="1">
+      <c r="A10" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B10" s="15">
+        <v>23.22</v>
+      </c>
+      <c r="C10" s="15">
+        <v>14.46</v>
+      </c>
+      <c r="D10" s="15">
+        <v>24.2</v>
+      </c>
+      <c r="E10" s="15">
+        <v>9.9</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="11" ht="22.5" customHeight="1">
+      <c r="G11" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="12" ht="22.5" customHeight="1">
+      <c r="G12" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="13" ht="22.5" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>165</v>
+      </c>
+      <c r="E13" s="24" t="s">
+        <v>184</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="14" ht="22.5" customHeight="1">
+      <c r="A14" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B14" s="20">
+        <f>MIN(C9:E9)</f>
+        <v>1.4</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="D14" s="11">
+        <f>MIN(C10:E10)</f>
+        <v>9.9</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="15" ht="22.5" customHeight="1">
+      <c r="A15" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="B15" s="20">
+        <f>MAX(C9:E9)</f>
+        <v>5.86</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="D15" s="11">
+        <f>MAX(C10:E10)</f>
+        <v>24.2</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="16" ht="22.5" customHeight="1">
+      <c r="A16" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="B16" s="20">
+        <f>AVERAGE(C9:E9)</f>
+        <v>3.09</v>
+      </c>
+      <c r="C16" s="20"/>
+      <c r="D16" s="11">
+        <f>AVERAGE(C10:E10)</f>
+        <v>16.18666667</v>
+      </c>
+    </row>
+    <row r="17" ht="22.5" customHeight="1">
+      <c r="A17" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="B17" s="20">
+        <f>MEDIAN(C9:E9)</f>
+        <v>2.01</v>
+      </c>
+      <c r="C17" s="20"/>
+      <c r="D17" s="11">
+        <f>MEDIAN(C10:E10)</f>
+        <v>14.46</v>
+      </c>
+    </row>
+    <row r="20" ht="22.5" customHeight="1">
+      <c r="A20" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B20" s="26" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="21" ht="22.5" customHeight="1">
+      <c r="A21" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B21" s="27">
+        <v>2.01</v>
+      </c>
+    </row>
+    <row r="22" ht="22.5" customHeight="1">
+      <c r="A22" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B22" s="28">
+        <f>B20*B21</f>
+        <v>5030.628</v>
+      </c>
+    </row>
+    <row r="23" ht="22.5" customHeight="1">
+      <c r="A23" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B23" s="28">
+        <f>B22+'Historical Financials'!E9-'Historical Financials'!E10</f>
+        <v>32498.128</v>
+      </c>
+    </row>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="A24" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="B24" s="29">
+        <v>14.46</v>
+      </c>
+    </row>
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="B25" s="30">
+        <v>498.7</v>
+      </c>
+    </row>
+    <row r="26" ht="22.5" customHeight="1">
+      <c r="A26" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B26" s="28">
+        <f>B24*B25</f>
+        <v>7211.202</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
+  <tableParts count="5">
+    <tablePart r:id="rId9"/>
+    <tablePart r:id="rId10"/>
+    <tablePart r:id="rId11"/>
+    <tablePart r:id="rId12"/>
+    <tablePart r:id="rId13"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="17.13"/>
+    <col customWidth="1" min="2" max="2" width="27.38"/>
+    <col customWidth="1" min="3" max="3" width="20.5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22.5" customHeight="1">
+      <c r="A1" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2" ht="22.5" customHeight="1">
+      <c r="A2" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B2" s="4">
+        <v>4620.0</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3" ht="22.5" customHeight="1">
+      <c r="A3" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B3" s="21">
+        <v>32498.0</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="4" ht="22.5" customHeight="1">
+      <c r="A4" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B4" s="21">
+        <v>7211.0</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B5" s="21">
+        <f>MEDIAN(B3,B4)</f>
+        <v>19854.5</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>171</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId5"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>